<commit_message>
UADEV-22214: added plan data logic and sample data
</commit_message>
<xml_diff>
--- a/BaseDocuments/flatwire tables.xlsx
+++ b/BaseDocuments/flatwire tables.xlsx
@@ -1,52 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30117"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nagarro-my.sharepoint.com/personal/shray_anand_nagarro_com/Documents/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="8_{9319DE46-1521-4FD6-B515-2DBCE7723D00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6BEF1961-31AC-48A7-ABFE-CE0DD48A9D6B}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="6" activeTab="7" xr2:uid="{B633ABBD-D7EC-4989-85E3-C4EFD5A554BD}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Drawer" sheetId="3" r:id="rId1"/>
-    <sheet name="Edger" sheetId="4" r:id="rId2"/>
-    <sheet name="RollerInfo" sheetId="5" r:id="rId3"/>
-    <sheet name="SpoolConfiguration" sheetId="6" r:id="rId4"/>
-    <sheet name="SpoolCoilMapping" sheetId="8" r:id="rId5"/>
-    <sheet name="Spool" sheetId="7" r:id="rId6"/>
-    <sheet name="FlatLinePassSchedule" sheetId="2" r:id="rId7"/>
-    <sheet name="FlatLineProcessing" sheetId="1" r:id="rId8"/>
+    <sheet sheetId="1" name="Drawer" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Edger" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="RollerInfo" state="visible" r:id="rId6"/>
+    <sheet sheetId="4" name="SpoolConfiguration" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="SpoolCoilMapping" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="Spool" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="FlatLinePassSchedule" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="FlatLineProcessing" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="SMP Scenarios" state="visible" r:id="rId12"/>
+    <sheet sheetId="10" name="FLP Mock" state="visible" r:id="rId13"/>
   </sheets>
-  <calcPr calcId="191028"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="71">
   <si>
     <t>Id</t>
   </si>
@@ -159,12 +133,27 @@
     <t>CoilOrderPlanId</t>
   </si>
   <si>
+    <t>IncomingCoilNo</t>
+  </si>
+  <si>
     <t>OnGaugeWeight</t>
   </si>
   <si>
     <t>OutputOD</t>
   </si>
   <si>
+    <t>PassScheduleId?</t>
+  </si>
+  <si>
+    <t>FlatLineComponent</t>
+  </si>
+  <si>
+    <t>Drawer /Stand</t>
+  </si>
+  <si>
+    <t>ComponentSeqNo</t>
+  </si>
+  <si>
     <t>OutputID</t>
   </si>
   <si>
@@ -177,29 +166,86 @@
     <t>StartGauge</t>
   </si>
   <si>
+    <t>MinTargetGauge</t>
+  </si>
+  <si>
     <t>TargetGauge</t>
   </si>
   <si>
-    <t>IncomingCoilNo</t>
-  </si>
-  <si>
-    <t>PassScheduleId</t>
+    <t>MaxTargetGauge</t>
+  </si>
+  <si>
+    <t>InputShape</t>
+  </si>
+  <si>
+    <t>Round/Flat</t>
+  </si>
+  <si>
+    <t>InputType</t>
+  </si>
+  <si>
+    <t>Rod/Wire</t>
+  </si>
+  <si>
+    <t>OutputShape</t>
+  </si>
+  <si>
+    <t>OutputType</t>
+  </si>
+  <si>
+    <t>Temper</t>
   </si>
   <si>
     <t>BackToStock</t>
+  </si>
+  <si>
+    <t>SMP / Process</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Flatten</t>
+  </si>
+  <si>
+    <t>FL2/FL3</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>FL1</t>
+  </si>
+  <si>
+    <t>Anneal</t>
+  </si>
+  <si>
+    <t>Furnace</t>
+  </si>
+  <si>
+    <t>FL2</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>Draw</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -252,44 +298,44 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
@@ -317,31 +363,14 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
         <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
+        <a:font script="Hans" typeface="宋体"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
@@ -369,23 +398,6 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -397,136 +409,180 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="35000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
+                <a:tint val="100000"/>
                 <a:shade val="100000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
-            <a:schemeClr val="phClr"/>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="40000">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
     <a:lnDef>
       <a:spPr/>
       <a:bodyPr/>
@@ -548,424 +604,863 @@
     </a:lnDef>
   </a:objectDefaults>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD0542F0-C70D-4763-9E68-3F239047699C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="23.28515625" customWidth="1"/>
+    <col min="1" max="1" width="23.285714285714285" customWidth="1"/>
+    <col min="2" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A27"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="26" width="13.571428571428571" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>58</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09B096A1-80AB-4BBF-9944-FCA6252F3059}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="24" width="13.571428571428571" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9A1B764-43C4-4BDB-B8CE-80DE6F1ADDF6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="24" width="13.571428571428571" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C881391-ED0B-481E-ABBE-E2DA63F87D9F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" customWidth="1"/>
+    <col min="1" max="1" width="11.571428571428571" customWidth="1"/>
+    <col min="2" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:1">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:1">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:1">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:1">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:1">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0A0E830-FB69-43F4-9F35-7C0566895DF7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="24" width="13.571428571428571" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD661918-87FA-44CA-9893-F7EC914FC98E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>20</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A37F033A-65B3-4ED9-A4CD-8E7A2FCB9775}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:1">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:1">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:1">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:1">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="1:1">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:1">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>18</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8B5FB46-34B7-4287-A39B-05A70E621615}">
-  <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B27"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="22.85546875" customWidth="1"/>
-    <col min="2" max="2" width="30.5703125" customWidth="1"/>
+    <col min="1" max="1" width="22.857142857142858" customWidth="1"/>
+    <col min="2" max="2" width="30.571428571428573" customWidth="1"/>
+    <col min="3" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
-      <c r="A11" t="s">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
-      <c r="A12" t="s">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>40</v>
       </c>
-      <c r="B12" t="s">
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="13" spans="1:2">
-      <c r="A13" t="s">
+      <c r="B14" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
-      <c r="A14" t="s">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
-      <c r="A15" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="17" spans="1:1">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="18" spans="1:1">
+      <c r="B17" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>46</v>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>51</v>
+      </c>
+      <c r="B22" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>53</v>
+      </c>
+      <c r="B23" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>55</v>
+      </c>
+      <c r="B24" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>56</v>
+      </c>
+      <c r="B25" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E30"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="37.857142857142854" customWidth="1"/>
+    <col min="2" max="26" width="13.571428571428571" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>61</v>
+      </c>
+      <c r="D8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>65</v>
+      </c>
+      <c r="D9" t="s">
+        <v>65</v>
+      </c>
+      <c r="E9" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" t="s">
+        <v>61</v>
+      </c>
+      <c r="E10" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>61</v>
+      </c>
+      <c r="D14" t="s">
+        <v>61</v>
+      </c>
+      <c r="E14" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>65</v>
+      </c>
+      <c r="D15" t="s">
+        <v>65</v>
+      </c>
+      <c r="E15" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>61</v>
+      </c>
+      <c r="D16" t="s">
+        <v>61</v>
+      </c>
+      <c r="E16" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>61</v>
+      </c>
+      <c r="D20" t="s">
+        <v>61</v>
+      </c>
+      <c r="E20" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>65</v>
+      </c>
+      <c r="D21" t="s">
+        <v>65</v>
+      </c>
+      <c r="E21" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>61</v>
+      </c>
+      <c r="D22" t="s">
+        <v>61</v>
+      </c>
+      <c r="E22" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>70</v>
+      </c>
+      <c r="D27" t="s">
+        <v>61</v>
+      </c>
+      <c r="E27" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>61</v>
+      </c>
+      <c r="D28" t="s">
+        <v>65</v>
+      </c>
+      <c r="E28" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>65</v>
+      </c>
+      <c r="D29" t="s">
+        <v>61</v>
+      </c>
+      <c r="E29" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>